<commit_message>
thêm biểu mẫu khoảng cách phù hợp hơn
</commit_message>
<xml_diff>
--- a/backend/templates/phieu-xuat-kho-template/warehouse-release-form-template.xlsx
+++ b/backend/templates/phieu-xuat-kho-template/warehouse-release-form-template.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\phamv\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B7C129C-FD1B-4870-9D95-A0C6A316510B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9B54452-0A9C-4874-AAC4-BCCF47CA5228}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-1545" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Page1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913" calcOnSave="0"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -613,6 +613,12 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -622,29 +628,23 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -965,10 +965,13 @@
     <col min="17" max="19" width="3.42578125" style="1" customWidth="1"/>
     <col min="20" max="22" width="3.85546875" style="1" customWidth="1"/>
     <col min="23" max="23" width="0.42578125" style="1" customWidth="1"/>
-    <col min="24" max="25" width="4.140625" style="1" customWidth="1"/>
-    <col min="26" max="26" width="4.85546875" style="1" customWidth="1"/>
-    <col min="27" max="30" width="4.140625" style="1" customWidth="1"/>
-    <col min="31" max="31" width="4.5703125" style="1" customWidth="1"/>
+    <col min="24" max="24" width="6.7109375" style="1" customWidth="1"/>
+    <col min="25" max="25" width="6.140625" style="1" customWidth="1"/>
+    <col min="26" max="27" width="6.7109375" style="1" customWidth="1"/>
+    <col min="28" max="28" width="4.42578125" style="1" customWidth="1"/>
+    <col min="29" max="29" width="6.42578125" style="1" customWidth="1"/>
+    <col min="30" max="30" width="4.85546875" style="1" customWidth="1"/>
+    <col min="31" max="31" width="8.42578125" style="1" customWidth="1"/>
     <col min="32" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
@@ -1130,40 +1133,40 @@
       <c r="A14" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B14" s="36" t="s">
+      <c r="B14" s="34" t="s">
         <v>10</v>
       </c>
-      <c r="C14" s="37"/>
-      <c r="D14" s="36" t="s">
+      <c r="C14" s="36"/>
+      <c r="D14" s="34" t="s">
         <v>11</v>
       </c>
-      <c r="E14" s="39"/>
-      <c r="F14" s="39"/>
-      <c r="G14" s="37"/>
-      <c r="H14" s="36" t="s">
+      <c r="E14" s="35"/>
+      <c r="F14" s="35"/>
+      <c r="G14" s="36"/>
+      <c r="H14" s="34" t="s">
         <v>12</v>
       </c>
-      <c r="I14" s="37"/>
-      <c r="J14" s="36" t="s">
+      <c r="I14" s="36"/>
+      <c r="J14" s="34" t="s">
         <v>13</v>
       </c>
-      <c r="K14" s="37"/>
-      <c r="L14" s="36" t="s">
+      <c r="K14" s="36"/>
+      <c r="L14" s="34" t="s">
         <v>14</v>
       </c>
-      <c r="M14" s="37"/>
+      <c r="M14" s="36"/>
       <c r="N14" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="O14" s="36" t="s">
+      <c r="O14" s="34" t="s">
         <v>22</v>
       </c>
-      <c r="P14" s="37"/>
-      <c r="Q14" s="36" t="s">
+      <c r="P14" s="36"/>
+      <c r="Q14" s="34" t="s">
         <v>21</v>
       </c>
-      <c r="R14" s="39"/>
-      <c r="S14" s="37"/>
+      <c r="R14" s="35"/>
+      <c r="S14" s="36"/>
       <c r="T14" s="40" t="s">
         <v>20</v>
       </c>
@@ -1176,51 +1179,51 @@
       <c r="Y14" s="40"/>
       <c r="Z14" s="40"/>
       <c r="AA14" s="40"/>
-      <c r="AB14" s="36" t="s">
+      <c r="AB14" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="AC14" s="39"/>
-      <c r="AD14" s="39"/>
-      <c r="AE14" s="37"/>
+      <c r="AC14" s="35"/>
+      <c r="AD14" s="35"/>
+      <c r="AE14" s="36"/>
     </row>
     <row r="15" spans="1:31" s="7" customFormat="1" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A15" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="B15" s="34" t="s">
+      <c r="B15" s="37" t="s">
         <v>26</v>
       </c>
-      <c r="C15" s="35"/>
-      <c r="D15" s="34" t="s">
+      <c r="C15" s="39"/>
+      <c r="D15" s="37" t="s">
         <v>27</v>
       </c>
       <c r="E15" s="38"/>
       <c r="F15" s="38"/>
-      <c r="G15" s="35"/>
-      <c r="H15" s="34" t="s">
+      <c r="G15" s="39"/>
+      <c r="H15" s="37" t="s">
         <v>28</v>
       </c>
-      <c r="I15" s="35"/>
-      <c r="J15" s="34" t="s">
+      <c r="I15" s="39"/>
+      <c r="J15" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="K15" s="35"/>
-      <c r="L15" s="34" t="s">
+      <c r="K15" s="39"/>
+      <c r="L15" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="M15" s="35"/>
+      <c r="M15" s="39"/>
       <c r="N15" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="O15" s="34">
+      <c r="O15" s="37">
         <v>1</v>
       </c>
-      <c r="P15" s="35"/>
-      <c r="Q15" s="34">
+      <c r="P15" s="39"/>
+      <c r="Q15" s="37">
         <v>2</v>
       </c>
       <c r="R15" s="38"/>
-      <c r="S15" s="35"/>
+      <c r="S15" s="39"/>
       <c r="T15" s="41">
         <v>3</v>
       </c>
@@ -1232,45 +1235,45 @@
       <c r="Y15" s="41"/>
       <c r="Z15" s="41"/>
       <c r="AA15" s="41"/>
-      <c r="AB15" s="34">
+      <c r="AB15" s="37">
         <v>3</v>
       </c>
       <c r="AC15" s="38"/>
       <c r="AD15" s="38"/>
-      <c r="AE15" s="35"/>
+      <c r="AE15" s="39"/>
     </row>
     <row r="16" spans="1:31" s="9" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="11"/>
-      <c r="B16" s="29"/>
-      <c r="C16" s="30"/>
-      <c r="D16" s="29"/>
-      <c r="E16" s="30"/>
-      <c r="F16" s="30"/>
-      <c r="G16" s="31"/>
-      <c r="H16" s="29"/>
-      <c r="I16" s="31"/>
-      <c r="J16" s="30"/>
-      <c r="K16" s="31"/>
-      <c r="L16" s="29"/>
-      <c r="M16" s="31"/>
+      <c r="B16" s="31"/>
+      <c r="C16" s="32"/>
+      <c r="D16" s="31"/>
+      <c r="E16" s="32"/>
+      <c r="F16" s="32"/>
+      <c r="G16" s="33"/>
+      <c r="H16" s="31"/>
+      <c r="I16" s="33"/>
+      <c r="J16" s="32"/>
+      <c r="K16" s="33"/>
+      <c r="L16" s="31"/>
+      <c r="M16" s="33"/>
       <c r="N16" s="11"/>
-      <c r="O16" s="32"/>
-      <c r="P16" s="33"/>
-      <c r="Q16" s="29"/>
-      <c r="R16" s="30"/>
-      <c r="S16" s="31"/>
-      <c r="T16" s="29"/>
-      <c r="U16" s="30"/>
-      <c r="V16" s="31"/>
+      <c r="O16" s="29"/>
+      <c r="P16" s="30"/>
+      <c r="Q16" s="31"/>
+      <c r="R16" s="32"/>
+      <c r="S16" s="33"/>
+      <c r="T16" s="31"/>
+      <c r="U16" s="32"/>
+      <c r="V16" s="33"/>
       <c r="W16" s="11"/>
-      <c r="X16" s="29"/>
-      <c r="Y16" s="30"/>
-      <c r="Z16" s="30"/>
-      <c r="AA16" s="31"/>
-      <c r="AB16" s="29"/>
-      <c r="AC16" s="30"/>
-      <c r="AD16" s="30"/>
-      <c r="AE16" s="31"/>
+      <c r="X16" s="31"/>
+      <c r="Y16" s="32"/>
+      <c r="Z16" s="32"/>
+      <c r="AA16" s="33"/>
+      <c r="AB16" s="31"/>
+      <c r="AC16" s="32"/>
+      <c r="AD16" s="32"/>
+      <c r="AE16" s="33"/>
     </row>
     <row r="17" spans="1:31" s="9" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="12"/>
@@ -4635,7 +4638,6 @@
     <mergeCell ref="L60:M60"/>
     <mergeCell ref="O60:P60"/>
     <mergeCell ref="Q60:S60"/>
-    <mergeCell ref="T58:V58"/>
     <mergeCell ref="X58:AA58"/>
     <mergeCell ref="T114:V114"/>
     <mergeCell ref="X114:AA114"/>
@@ -4661,6 +4663,12 @@
     <mergeCell ref="O113:P113"/>
     <mergeCell ref="Q113:S113"/>
     <mergeCell ref="AB58:AE58"/>
+    <mergeCell ref="B102:C102"/>
+    <mergeCell ref="D102:G102"/>
+    <mergeCell ref="H102:I102"/>
+    <mergeCell ref="J102:K102"/>
+    <mergeCell ref="L102:M102"/>
+    <mergeCell ref="O102:P102"/>
     <mergeCell ref="T57:V57"/>
     <mergeCell ref="X57:AA57"/>
     <mergeCell ref="AB57:AE57"/>
@@ -4692,12 +4700,7 @@
     <mergeCell ref="O61:P61"/>
     <mergeCell ref="Q61:S61"/>
     <mergeCell ref="Q57:S57"/>
-    <mergeCell ref="B102:C102"/>
-    <mergeCell ref="D102:G102"/>
-    <mergeCell ref="H102:I102"/>
-    <mergeCell ref="J102:K102"/>
-    <mergeCell ref="L102:M102"/>
-    <mergeCell ref="O102:P102"/>
+    <mergeCell ref="T58:V58"/>
     <mergeCell ref="Q102:S102"/>
     <mergeCell ref="T62:V62"/>
     <mergeCell ref="X62:AA62"/>
@@ -4724,6 +4727,12 @@
     <mergeCell ref="H67:I67"/>
     <mergeCell ref="J67:K67"/>
     <mergeCell ref="L67:M67"/>
+    <mergeCell ref="O67:P67"/>
+    <mergeCell ref="Q67:S67"/>
+    <mergeCell ref="T65:V65"/>
+    <mergeCell ref="X65:AA65"/>
+    <mergeCell ref="AB65:AE65"/>
+    <mergeCell ref="B66:C66"/>
     <mergeCell ref="B109:C109"/>
     <mergeCell ref="B110:C110"/>
     <mergeCell ref="B111:C111"/>
@@ -5048,6 +5057,10 @@
     <mergeCell ref="AB55:AE55"/>
     <mergeCell ref="X54:AA54"/>
     <mergeCell ref="AB54:AE54"/>
+    <mergeCell ref="T45:V45"/>
+    <mergeCell ref="X45:AA45"/>
+    <mergeCell ref="AB45:AE45"/>
+    <mergeCell ref="AB41:AE41"/>
     <mergeCell ref="B52:C52"/>
     <mergeCell ref="D52:G52"/>
     <mergeCell ref="H52:I52"/>
@@ -5072,6 +5085,14 @@
     <mergeCell ref="J41:K41"/>
     <mergeCell ref="L41:M41"/>
     <mergeCell ref="O41:P41"/>
+    <mergeCell ref="AB42:AE42"/>
+    <mergeCell ref="B43:C43"/>
+    <mergeCell ref="D43:G43"/>
+    <mergeCell ref="H43:I43"/>
+    <mergeCell ref="J43:K43"/>
+    <mergeCell ref="L43:M43"/>
+    <mergeCell ref="O43:P43"/>
+    <mergeCell ref="Q45:S45"/>
     <mergeCell ref="B38:C38"/>
     <mergeCell ref="D38:G38"/>
     <mergeCell ref="H38:I38"/>
@@ -5089,17 +5110,6 @@
     <mergeCell ref="Q42:S42"/>
     <mergeCell ref="T42:V42"/>
     <mergeCell ref="X42:AA42"/>
-    <mergeCell ref="AB42:AE42"/>
-    <mergeCell ref="B43:C43"/>
-    <mergeCell ref="D43:G43"/>
-    <mergeCell ref="H43:I43"/>
-    <mergeCell ref="J43:K43"/>
-    <mergeCell ref="L43:M43"/>
-    <mergeCell ref="O43:P43"/>
-    <mergeCell ref="Q45:S45"/>
-    <mergeCell ref="T45:V45"/>
-    <mergeCell ref="X45:AA45"/>
-    <mergeCell ref="AB45:AE45"/>
     <mergeCell ref="B39:C39"/>
     <mergeCell ref="D39:G39"/>
     <mergeCell ref="H39:I39"/>
@@ -5109,7 +5119,6 @@
     <mergeCell ref="Q41:S41"/>
     <mergeCell ref="T41:V41"/>
     <mergeCell ref="X41:AA41"/>
-    <mergeCell ref="AB41:AE41"/>
     <mergeCell ref="B42:C42"/>
     <mergeCell ref="D42:G42"/>
     <mergeCell ref="H42:I42"/>
@@ -5223,12 +5232,6 @@
     <mergeCell ref="L64:M64"/>
     <mergeCell ref="O64:P64"/>
     <mergeCell ref="Q64:S64"/>
-    <mergeCell ref="O67:P67"/>
-    <mergeCell ref="Q67:S67"/>
-    <mergeCell ref="T65:V65"/>
-    <mergeCell ref="X65:AA65"/>
-    <mergeCell ref="AB65:AE65"/>
-    <mergeCell ref="B66:C66"/>
     <mergeCell ref="D66:G66"/>
     <mergeCell ref="H66:I66"/>
     <mergeCell ref="J66:K66"/>
@@ -5569,7 +5572,7 @@
     <mergeCell ref="O97:P97"/>
     <mergeCell ref="Q97:S97"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>